<commit_message>
chore(ND-00): referenzdaten und headless-laufskript ergaenzen
* Spin-Off Data.xlsx - kuratierte Liste, die apply_spinoffs auswertet
  (3 Eintraege; Sandoz aus Novartis ist der einzige Schweizer Fall)
* Sanktionslisten (Bloomberg-Auszug, WM Daten) als Referenz. Bewusst
  NICHT eingelesen: der Screen laeuft spaeter ueber In-Eligible.xlsx.
* run_eupool.py - Europe-Pooled ohne Streamlit, fuer lange Laeufe
* aktualisierte Referenztabellen (Classification, Selection Dates,
  In-Eligible, Country Classification, China Inclusion Factor)
</commit_message>
<xml_diff>
--- a/China Inclusion Factor.xlsx
+++ b/China Inclusion Factor.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Geteilte Ablagen\NaroIX - Index Management\Framework\Rebalancing_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nico\naroix\NaroIX-Benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F9F09A-1577-4F34-AA1E-1C8640CDC8B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26635A7D-F538-437F-BD6D-94C99EF2C0BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-13860" yWindow="-16308" windowWidth="29016" windowHeight="15696" xr2:uid="{24FF59A1-7234-4942-98D7-B7BE7DF6F0AC}"/>
   </bookViews>
@@ -568,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA481E37-1CE1-49C4-A8D4-417DADDFB568}">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" style="1" bestFit="1" customWidth="1"/>
@@ -959,6 +959,22 @@
         <v>0.2</v>
       </c>
     </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>46162</v>
+      </c>
+      <c r="B49" s="2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>46253</v>
+      </c>
+      <c r="B50" s="2">
+        <v>0.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>